<commit_message>
product typ (green and burnt) status improvement
</commit_message>
<xml_diff>
--- a/log_procurement.backup.xlsx
+++ b/log_procurement.backup.xlsx
@@ -485,7 +485,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -509,74 +509,22 @@
         <v>Radiata Pine</v>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>User-added species</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Eucalyptus</v>
-      </c>
-      <c r="C3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D3" t="str">
-        <v>User-added species</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>test</v>
-      </c>
-      <c r="C4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" t="str">
-        <v>User-added species</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>dsfd</v>
-      </c>
-      <c r="C5" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" t="str">
-        <v>User-added species</v>
+        <v>Standard plantation softwood</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H65"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:H56"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1542,7 +1490,7 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B38" t="str">
         <v/>
@@ -1554,7 +1502,7 @@
         <v>test</v>
       </c>
       <c r="E38" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F38" t="str">
         <v>SA Grade</v>
@@ -1568,7 +1516,7 @@
     </row>
     <row r="39">
       <c r="A39">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B39" t="str">
         <v/>
@@ -1580,7 +1528,7 @@
         <v>test</v>
       </c>
       <c r="E39" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F39" t="str">
         <v>A Grade</v>
@@ -1594,7 +1542,7 @@
     </row>
     <row r="40">
       <c r="A40">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B40" t="str">
         <v/>
@@ -1606,7 +1554,7 @@
         <v>test</v>
       </c>
       <c r="E40" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F40" t="str">
         <v>K Grade</v>
@@ -1620,7 +1568,7 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B41" t="str">
         <v/>
@@ -1632,7 +1580,7 @@
         <v>test</v>
       </c>
       <c r="E41" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F41" t="str">
         <v>KI Grade</v>
@@ -1646,7 +1594,7 @@
     </row>
     <row r="42">
       <c r="A42">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B42" t="str">
         <v/>
@@ -1658,7 +1606,7 @@
         <v>test</v>
       </c>
       <c r="E42" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F42" t="str">
         <v>MP Grade</v>
@@ -1672,7 +1620,7 @@
     </row>
     <row r="43">
       <c r="A43">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="B43" t="str">
         <v/>
@@ -1681,13 +1629,13 @@
         <v/>
       </c>
       <c r="D43" t="str">
-        <v>test</v>
+        <v>dsfd</v>
       </c>
       <c r="E43" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F43" t="str">
-        <v>Big MP</v>
+        <v>SA Grade</v>
       </c>
       <c r="G43" t="b">
         <v>1</v>
@@ -1698,7 +1646,7 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B44" t="str">
         <v/>
@@ -1707,13 +1655,13 @@
         <v/>
       </c>
       <c r="D44" t="str">
-        <v>test</v>
+        <v>dsfd</v>
       </c>
       <c r="E44" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F44" t="str">
-        <v>Pulp</v>
+        <v>A Grade</v>
       </c>
       <c r="G44" t="b">
         <v>1</v>
@@ -1724,7 +1672,7 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="B45" t="str">
         <v/>
@@ -1733,13 +1681,13 @@
         <v/>
       </c>
       <c r="D45" t="str">
-        <v>test</v>
+        <v>dsfd</v>
       </c>
       <c r="E45" t="str">
         <v>Burnt</v>
       </c>
       <c r="F45" t="str">
-        <v>SA Grade</v>
+        <v>K Grade</v>
       </c>
       <c r="G45" t="b">
         <v>1</v>
@@ -1750,7 +1698,7 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="B46" t="str">
         <v/>
@@ -1759,13 +1707,13 @@
         <v/>
       </c>
       <c r="D46" t="str">
-        <v>test</v>
+        <v>dsfd</v>
       </c>
       <c r="E46" t="str">
         <v>Burnt</v>
       </c>
       <c r="F46" t="str">
-        <v>A Grade</v>
+        <v>KI Grade</v>
       </c>
       <c r="G46" t="b">
         <v>1</v>
@@ -1776,7 +1724,7 @@
     </row>
     <row r="47">
       <c r="A47">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="B47" t="str">
         <v/>
@@ -1785,13 +1733,13 @@
         <v/>
       </c>
       <c r="D47" t="str">
-        <v>test</v>
+        <v>dsfd</v>
       </c>
       <c r="E47" t="str">
         <v>Burnt</v>
       </c>
       <c r="F47" t="str">
-        <v>K Grade</v>
+        <v>MP Grade</v>
       </c>
       <c r="G47" t="b">
         <v>1</v>
@@ -1802,475 +1750,241 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="B48" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C48" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D48" t="str">
-        <v>test</v>
+        <v/>
       </c>
       <c r="E48" t="str">
-        <v>Burnt</v>
+        <v>Green</v>
       </c>
       <c r="F48" t="str">
-        <v>KI Grade</v>
+        <v>A</v>
       </c>
       <c r="G48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H48" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
+        <v>User-added grade</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="B49" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C49" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D49" t="str">
-        <v>test</v>
+        <v/>
       </c>
       <c r="E49" t="str">
         <v>Burnt</v>
       </c>
       <c r="F49" t="str">
-        <v>MP Grade</v>
+        <v>A</v>
       </c>
       <c r="G49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H49" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
+        <v>User-added grade</v>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="B50" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C50" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D50" t="str">
-        <v>dsfd</v>
+        <v/>
       </c>
       <c r="E50" t="str">
         <v>Green</v>
       </c>
       <c r="F50" t="str">
-        <v>SA Grade</v>
+        <v>K</v>
       </c>
       <c r="G50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H50" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
+        <v>User-added grade</v>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B51" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C51" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D51" t="str">
-        <v>dsfd</v>
+        <v/>
       </c>
       <c r="E51" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F51" t="str">
-        <v>A Grade</v>
+        <v>K</v>
       </c>
       <c r="G51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H51" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
+        <v>User-added grade</v>
       </c>
     </row>
     <row r="52">
       <c r="A52">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="B52" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C52" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D52" t="str">
-        <v>dsfd</v>
+        <v/>
       </c>
       <c r="E52" t="str">
         <v>Green</v>
       </c>
       <c r="F52" t="str">
-        <v>K Grade</v>
+        <v>SA</v>
       </c>
       <c r="G52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H52" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
+        <v>User-added grade</v>
       </c>
     </row>
     <row r="53">
       <c r="A53">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B53" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C53" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D53" t="str">
-        <v>dsfd</v>
+        <v/>
       </c>
       <c r="E53" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F53" t="str">
-        <v>KI Grade</v>
+        <v>SA</v>
       </c>
       <c r="G53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H53" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
+        <v>User-added grade</v>
       </c>
     </row>
     <row r="54">
       <c r="A54">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="B54" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C54" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D54" t="str">
-        <v>dsfd</v>
+        <v/>
       </c>
       <c r="E54" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F54" t="str">
-        <v>MP Grade</v>
+        <v>BURNT</v>
       </c>
       <c r="G54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H54" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
+        <v>User-added grade</v>
       </c>
     </row>
     <row r="55">
       <c r="A55">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="B55" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C55" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D55" t="str">
-        <v>dsfd</v>
+        <v/>
       </c>
       <c r="E55" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F55" t="str">
-        <v>Big MP</v>
+        <v>TEST</v>
       </c>
       <c r="G55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H55" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
+        <v>User-added grade</v>
       </c>
     </row>
     <row r="56">
       <c r="A56">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="B56" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="C56" t="str">
-        <v/>
+        <v>HVP</v>
       </c>
       <c r="D56" t="str">
-        <v>dsfd</v>
+        <v/>
       </c>
       <c r="E56" t="str">
-        <v>Green</v>
+        <v>Burnt</v>
       </c>
       <c r="F56" t="str">
-        <v>Pulp</v>
+        <v>1</v>
       </c>
       <c r="G56" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H56" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57">
-        <v>56</v>
-      </c>
-      <c r="B57" t="str">
-        <v/>
-      </c>
-      <c r="C57" t="str">
-        <v/>
-      </c>
-      <c r="D57" t="str">
-        <v>dsfd</v>
-      </c>
-      <c r="E57" t="str">
-        <v>Burnt</v>
-      </c>
-      <c r="F57" t="str">
-        <v>SA Grade</v>
-      </c>
-      <c r="G57" t="b">
-        <v>1</v>
-      </c>
-      <c r="H57" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58" t="str">
-        <v/>
-      </c>
-      <c r="C58" t="str">
-        <v/>
-      </c>
-      <c r="D58" t="str">
-        <v>dsfd</v>
-      </c>
-      <c r="E58" t="str">
-        <v>Burnt</v>
-      </c>
-      <c r="F58" t="str">
-        <v>A Grade</v>
-      </c>
-      <c r="G58" t="b">
-        <v>1</v>
-      </c>
-      <c r="H58" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59">
-        <v>58</v>
-      </c>
-      <c r="B59" t="str">
-        <v/>
-      </c>
-      <c r="C59" t="str">
-        <v/>
-      </c>
-      <c r="D59" t="str">
-        <v>dsfd</v>
-      </c>
-      <c r="E59" t="str">
-        <v>Burnt</v>
-      </c>
-      <c r="F59" t="str">
-        <v>K Grade</v>
-      </c>
-      <c r="G59" t="b">
-        <v>1</v>
-      </c>
-      <c r="H59" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60">
-        <v>59</v>
-      </c>
-      <c r="B60" t="str">
-        <v/>
-      </c>
-      <c r="C60" t="str">
-        <v/>
-      </c>
-      <c r="D60" t="str">
-        <v>dsfd</v>
-      </c>
-      <c r="E60" t="str">
-        <v>Burnt</v>
-      </c>
-      <c r="F60" t="str">
-        <v>KI Grade</v>
-      </c>
-      <c r="G60" t="b">
-        <v>1</v>
-      </c>
-      <c r="H60" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61">
-        <v>60</v>
-      </c>
-      <c r="B61" t="str">
-        <v/>
-      </c>
-      <c r="C61" t="str">
-        <v/>
-      </c>
-      <c r="D61" t="str">
-        <v>dsfd</v>
-      </c>
-      <c r="E61" t="str">
-        <v>Burnt</v>
-      </c>
-      <c r="F61" t="str">
-        <v>MP Grade</v>
-      </c>
-      <c r="G61" t="b">
-        <v>1</v>
-      </c>
-      <c r="H61" t="str">
-        <v>Standard grade from Log Procurement reference PDF</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62">
-        <v>61</v>
-      </c>
-      <c r="B62" t="str">
-        <v>1</v>
-      </c>
-      <c r="C62" t="str">
-        <v>HVP</v>
-      </c>
-      <c r="D62" t="str">
-        <v/>
-      </c>
-      <c r="E62" t="str">
-        <v>Green</v>
-      </c>
-      <c r="F62" t="str">
-        <v>a</v>
-      </c>
-      <c r="G62" t="b">
-        <v>0</v>
-      </c>
-      <c r="H62" t="str">
-        <v>User-added grade</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63">
-        <v>62</v>
-      </c>
-      <c r="B63" t="str">
-        <v>1</v>
-      </c>
-      <c r="C63" t="str">
-        <v>HVP</v>
-      </c>
-      <c r="D63" t="str">
-        <v/>
-      </c>
-      <c r="E63" t="str">
-        <v>Green</v>
-      </c>
-      <c r="F63" t="str">
-        <v>b</v>
-      </c>
-      <c r="G63" t="b">
-        <v>0</v>
-      </c>
-      <c r="H63" t="str">
-        <v>User-added grade</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64">
-        <v>63</v>
-      </c>
-      <c r="B64" t="str">
-        <v>1</v>
-      </c>
-      <c r="C64" t="str">
-        <v>HVP</v>
-      </c>
-      <c r="D64" t="str">
-        <v/>
-      </c>
-      <c r="E64" t="str">
-        <v>Green</v>
-      </c>
-      <c r="F64" t="str">
-        <v>c</v>
-      </c>
-      <c r="G64" t="b">
-        <v>0</v>
-      </c>
-      <c r="H64" t="str">
-        <v>User-added grade</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65">
-        <v>64</v>
-      </c>
-      <c r="B65" t="str">
-        <v>1</v>
-      </c>
-      <c r="C65" t="str">
-        <v>HVP</v>
-      </c>
-      <c r="D65" t="str">
-        <v/>
-      </c>
-      <c r="E65" t="str">
-        <v>Green</v>
-      </c>
-      <c r="F65" t="str">
-        <v>d</v>
-      </c>
-      <c r="G65" t="b">
-        <v>0</v>
-      </c>
-      <c r="H65" t="str">
         <v>User-added grade</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H56"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2348,7 +2062,37 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:AB4"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" customWidth="1"/>
+    <col min="15" max="15" width="20.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="20.83203125" customWidth="1"/>
+    <col min="18" max="18" width="20.83203125" customWidth="1"/>
+    <col min="19" max="19" width="20.83203125" customWidth="1"/>
+    <col min="20" max="20" width="20.83203125" customWidth="1"/>
+    <col min="21" max="21" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="20.83203125" customWidth="1"/>
+    <col min="23" max="23" width="20.83203125" customWidth="1"/>
+    <col min="24" max="24" width="20.83203125" customWidth="1"/>
+    <col min="25" max="25" width="20.83203125" customWidth="1"/>
+    <col min="26" max="26" width="20.83203125" customWidth="1"/>
+    <col min="27" max="27" width="20.83203125" customWidth="1"/>
+    <col min="28" max="28" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2388,37 +2132,52 @@
         <v>EndDate</v>
       </c>
       <c r="M1" t="str">
+        <v>WeeklyEstimatedTonnes</v>
+      </c>
+      <c r="N1" t="str">
         <v>Status</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>AcceptanceDate</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>AcceptanceTime</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>AcceptanceMethod</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>AcceptedByPerson</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>AcceptanceNotes</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
+        <v>LogSpecFileID</v>
+      </c>
+      <c r="U1" t="str">
+        <v>LogSpecFileName</v>
+      </c>
+      <c r="V1" t="str">
+        <v>LogSpecFileType</v>
+      </c>
+      <c r="W1" t="str">
         <v>Notes</v>
       </c>
-      <c r="T1" t="str">
+      <c r="X1" t="str">
         <v>CreatedBy</v>
       </c>
-      <c r="U1" t="str">
+      <c r="Y1" t="str">
         <v>CreatedDate</v>
       </c>
-      <c r="V1" t="str">
+      <c r="Z1" t="str">
         <v>ChangedBy</v>
       </c>
-      <c r="W1" t="str">
+      <c r="AA1" t="str">
         <v>ChangedDate</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>ForceWeeklyForecast</v>
       </c>
     </row>
     <row r="2">
@@ -2428,10 +2187,10 @@
       <c r="B2" t="str">
         <v>PROC-0001</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
+      <c r="C2" t="str">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
         <v>1</v>
       </c>
       <c r="E2" t="str">
@@ -2443,6 +2202,9 @@
       <c r="G2" t="str">
         <v>PLANTATION</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
       <c r="I2" t="str">
         <v>KLJ</v>
       </c>
@@ -2456,37 +2218,52 @@
         <v>SAD</v>
       </c>
       <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
         <v>Draft</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>SDA</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>SA</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v>In Person</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>SAD</v>
-      </c>
-      <c r="R2" t="str">
-        <v>ASD</v>
       </c>
       <c r="S2" t="str">
         <v>ASD</v>
       </c>
       <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v>ASD</v>
+      </c>
+      <c r="X2" t="str">
         <v>Current User</v>
       </c>
-      <c r="U2" t="str">
+      <c r="Y2" t="str">
         <v>2026-09-15 00:52:10</v>
       </c>
-      <c r="V2" t="str">
+      <c r="Z2" t="str">
         <v>Current User</v>
       </c>
-      <c r="W2" t="str">
+      <c r="AA2" t="str">
         <v>2026-09-15 00:52:10</v>
+      </c>
+      <c r="AB2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2496,10 +2273,10 @@
       <c r="B3" t="str">
         <v>PROC-0002</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
+      <c r="C3" t="str">
+        <v>1</v>
+      </c>
+      <c r="D3" t="str">
         <v>1</v>
       </c>
       <c r="E3" t="str">
@@ -2511,6 +2288,9 @@
       <c r="G3" t="str">
         <v>SDF</v>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
       <c r="I3" t="str">
         <v>SDFSD</v>
       </c>
@@ -2524,51 +2304,164 @@
         <v>DSF</v>
       </c>
       <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
         <v>Draft</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>GFH</v>
       </c>
-      <c r="O3" t="str">
+      <c r="P3" t="str">
         <v>HGF</v>
       </c>
-      <c r="P3" t="str">
+      <c r="Q3" t="str">
         <v>Phone</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="R3" t="str">
         <v>GFH</v>
       </c>
-      <c r="R3" t="str">
+      <c r="S3" t="str">
         <v>GHF</v>
       </c>
-      <c r="S3" t="str">
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
         <v>FGH</v>
       </c>
-      <c r="T3" t="str">
+      <c r="X3" t="str">
         <v>Current User</v>
       </c>
-      <c r="U3" t="str">
+      <c r="Y3" t="str">
         <v>2026-09-15 00:54:11</v>
       </c>
-      <c r="V3" t="str">
+      <c r="Z3" t="str">
         <v>Current User</v>
       </c>
-      <c r="W3" t="str">
+      <c r="AA3" t="str">
         <v>2026-09-15 00:54:11</v>
       </c>
+      <c r="AB3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>HVP-0001</v>
+      </c>
+      <c r="C4" t="str">
+        <v>1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Coupe</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Radiata Pine</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4">
+        <v>3300</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Active</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>In Person</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v>Current User</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>2026-09-25 08:24:22</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>Current User</v>
+      </c>
+      <c r="AA4" t="str">
+        <v>2026-09-25 08:24:22</v>
+      </c>
+      <c r="AB4" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L5"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2593,15 +2486,18 @@
         <v>AgreedPricePerTonne</v>
       </c>
       <c r="H1" t="str">
+        <v>ResalePrice</v>
+      </c>
+      <c r="I1" t="str">
         <v>AgreedTonnes</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>DeliveredTonnes</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>RemainingTonnes</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -2628,13 +2524,19 @@
         <v>70</v>
       </c>
       <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
         <v>3000</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>0</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>3000</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -2660,13 +2562,19 @@
         <v>60</v>
       </c>
       <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
         <v>2000</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>0</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>2000</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -2692,20 +2600,62 @@
         <v>55</v>
       </c>
       <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
         <v>5000</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>0</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>5000</v>
       </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>HVP-0001</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Radiata Pine</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Green</v>
+      </c>
+      <c r="E5" t="str">
+        <v>A</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>